<commit_message>
added GDP growth rate as feature
</commit_message>
<xml_diff>
--- a/code/Created Files for Analysis/further_selected_indicators.xlsx
+++ b/code/Created Files for Analysis/further_selected_indicators.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,34 +601,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gini verfügbares Einkommen (post-tax/transfer)</t>
+          <t>BIP-Wachstumsrate (real)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SWIID-GINI-DISP</t>
+          <t>WB-WDI-NY-GDP-MKTP-KD-ZG</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SWIID v9.92 (Solt 2019)</t>
+          <t>World Development Indicators (World Bank), via WISE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Einkommensungleichheit nach Steuern und Transfers (0-100)</t>
+          <t>Jaehrliche Wachstumsrate des realen BIP (konstant 2015 USD), abgeleitet aus dem BIP-Niveau (Vorjahresvergleich, % p.a.)</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>98.3</v>
+        <v>99.2</v>
       </c>
       <c r="G6" t="n">
-        <v>92</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="7">
@@ -639,12 +639,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gini Markteinkommen (pre-tax/transfer)</t>
+          <t>Gini verfügbares Einkommen (post-tax/transfer)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SWIID-GINI-MKT</t>
+          <t>SWIID-GINI-DISP</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Einkommensungleichheit vor Steuern und Transfers (0-100)</t>
+          <t>Einkommensungleichheit nach Steuern und Transfers (0-100)</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -667,132 +667,165 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Leistungsbilanzsaldo</t>
+          <t>Gini Markteinkommen (pre-tax/transfer)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BN.CAB.XOKA.GD.ZS</t>
+          <t>SWIID-GINI-MKT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>World Development Indicators (World Bank)</t>
+          <t>SWIID v9.92 (Solt 2019)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Nettoglaeubiger- (+) oder Nettoschuldnerposition (-) gegenueber dem Ausland aus Gueter-, DL- und Einkommensverkehr (% des BIP)</t>
+          <t>Einkommensungleichheit vor Steuern und Transfers (0-100)</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>97.5</v>
+        <v>98.3</v>
       </c>
       <c r="G8" t="n">
-        <v>95.8</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Zentralstaatsverschuldung (CG Debt)</t>
+          <t>Leistungsbilanzsaldo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>IMF-GDD-CG</t>
+          <t>BN.CAB.XOKA.GD.ZS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>IMF Global Debt Database (Mbaye et al. 2018)</t>
+          <t>World Development Indicators (World Bank)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Schuldenstand des Zentralstaats (% des BIP)</t>
+          <t>Nettoglaeubiger- (+) oder Nettoschuldnerposition (-) gegenueber dem Ausland aus Gueter-, DL- und Einkommensverkehr (% des BIP)</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>90.8</v>
+        <v>97.5</v>
       </c>
       <c r="G9" t="n">
-        <v>90.09999999999999</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4.11</t>
+          <t>4.12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Staatsquote</t>
+          <t>Zentralstaatsverschuldung (CG Debt)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GC.XPN.TOTL.GD.ZS</t>
+          <t>IMF-GDD-CG</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>World Development Indicators (World Bank)</t>
+          <t>IMF Global Debt Database (Mbaye et al. 2018)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Gesamte Staatsausgaben inkl. Transfers (% des BIP)</t>
+          <t>Schuldenstand des Zentralstaats (% des BIP)</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>88.2</v>
+        <v>90.8</v>
       </c>
       <c r="G10" t="n">
-        <v>77.2</v>
+        <v>90.09999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Staatsquote</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GC.XPN.TOTL.GD.ZS</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>World Development Indicators (World Bank)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Gesamte Staatsausgaben inkl. Transfers (% des BIP)</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>77.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>4.6</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Breite Geldmenge (M2)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>FM.LBL.BMNY.GD.ZS</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>World Development Indicators (World Bank)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Bargeld, Sicht- und kurzfristige Spareinlagen (% des BIP)</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="F12" t="n">
         <v>83.2</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G12" t="n">
         <v>78.3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added GDP growth rate
</commit_message>
<xml_diff>
--- a/code/Created Files for Analysis/further_selected_indicators.xlsx
+++ b/code/Created Files for Analysis/further_selected_indicators.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Jaehrliche Veraenderung des Verbraucherpreisindex (% p.a.)</t>
+          <t>Jährliche Veränderung des Verbraucherpreisindex (% p.a.)</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -522,7 +522,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Verhaeltnis Nominal- zu Real-BIP: Preisniveauaenderung aller produzierten Gueter (% p.a.)</t>
+          <t>Verhältnis Nominal- zu Real-BIP: Preisniveauänderung aller produzierten Gueter (% p.a.)</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -588,7 +588,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Verhaeltnis Exportpreise zu Importpreisen (Index, 2015=100)</t>
+          <t>Verhältnis Exportpreise zu Importpreisen (Index, 2015=100)</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -611,17 +611,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>WB-WDI-NY-GDP-MKTP-KD-ZG</t>
+          <t>WB-WDI-GDP-ZG</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>World Development Indicators (World Bank), via WISE</t>
+          <t>Calculated from World Development Indicators (World Bank) Features</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Jaehrliche Wachstumsrate des realen BIP (konstant 2015 USD), abgeleitet aus dem BIP-Niveau (Vorjahresvergleich, % p.a.)</t>
+          <t>Jährliche Wachstumsrate des realen BIP (konstant 2015 USD), abgeleitet aus dem BIP-Niveau (Vorjahresvergleich, % p.a.)</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -720,7 +720,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Nettoglaeubiger- (+) oder Nettoschuldnerposition (-) gegenueber dem Ausland aus Gueter-, DL- und Einkommensverkehr (% des BIP)</t>
+          <t>Nettogläubiger- (+) oder Nettoschuldnerposition (-) gegenueber dem Ausland aus Gueter-, DL- und Einkommensverkehr (% des BIP)</t>
         </is>
       </c>
       <c r="F9" t="n">

</xml_diff>